<commit_message>
Oct 17, 2026, 12:08 PM
</commit_message>
<xml_diff>
--- a/Premier League 2026-2027.xlsx
+++ b/Premier League 2026-2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9DF7064-8706-40F9-879E-2BE952DE888E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE0F7A27-052C-4537-8141-8FCEC5168D6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="548" xr2:uid="{C0939FE1-FA46-4B9A-8CEA-6583A57696E8}"/>
   </bookViews>
@@ -3819,22 +3819,22 @@
         <v>90</v>
       </c>
       <c r="BW11">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="BX11">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="BY11">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="BZ11">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="CA11">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="CB11">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="CC11">
         <v>8</v>

</xml_diff>